<commit_message>
Feat:- Changes in resources file
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>Event_Name</t>
   </si>
@@ -191,7 +191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,11 @@
         <v>44</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
add logic reset button
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
   <si>
     <t>Event_Name</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>Dehradun Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Udaipur Swachhta Hi Seva</t>
   </si>
 </sst>
 </file>
@@ -209,7 +212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -522,6 +525,16 @@
         <v>50</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
changes in Excel and tamplete
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="54">
   <si>
     <t>Event_Name</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t>Faridabad Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Pune Swachhta Hi Seva</t>
   </si>
 </sst>
 </file>
@@ -215,7 +218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A65"/>
+  <dimension ref="A1:A66"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -543,6 +546,11 @@
         <v>52</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
youth profile image and duplicate template name
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="56">
   <si>
     <t>Event_Name</t>
   </si>
@@ -174,6 +174,12 @@
   </si>
   <si>
     <t>Pune Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Ranchi Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Nagpur Swachhta Hi Seva</t>
   </si>
 </sst>
 </file>
@@ -218,7 +224,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A66"/>
+  <dimension ref="A1:A69"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -551,6 +557,21 @@
         <v>53</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="0">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix workflow email and count configuration
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="59">
   <si>
     <t>Event_Name</t>
   </si>
@@ -183,6 +183,12 @@
   </si>
   <si>
     <t>Noida Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Jaipur Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Patna Swachhta Hi Seva</t>
   </si>
 </sst>
 </file>
@@ -227,7 +233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A70"/>
+  <dimension ref="A1:A73"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -580,6 +586,21 @@
         <v>56</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s" s="0">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
changes in two files only
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
   <si>
     <t>Event_Name</t>
   </si>
@@ -233,7 +233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A73"/>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -601,6 +601,11 @@
         <v>58</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
add email in the prod
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="59">
   <si>
     <t>Event_Name</t>
   </si>
@@ -233,7 +233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A75"/>
+  <dimension ref="A1:A76"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -611,6 +611,11 @@
         <v>50</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update resource files and add ReadExcel utility
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="63">
   <si>
     <t>Event_Name</t>
   </si>
@@ -245,7 +245,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A81"/>
+  <dimension ref="A1:A82"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -653,6 +653,11 @@
         <v>48</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: set thread-count to 3 for parallel VO execution + update resources
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="63">
   <si>
     <t>Event_Name</t>
   </si>
@@ -245,7 +245,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A82"/>
+  <dimension ref="A1:A83"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -658,6 +658,11 @@
         <v>48</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>